<commit_message>
Expose door-pair drag and use it everywhere the total demand is built
The previous commit made the corrected total add both doors, but the
report breakdown, the demand table, the frontend composition chart and
chapter 18 still summed one door, and the web e2e test pinned the old
max speed (2.39 kn, now 2.28 kn).

- DoorStage.rig_drag_kgf = DOORS_PER_RIG · forces.drag_kgf; warps stage,
  report charts/tables and web series use it.
- Web: result type, recorded API fixture and unit/e2e expectations
  refreshed; examples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GxmE171J19C1A6ZvcYULfz
</commit_message>
<xml_diff>
--- a/examples/fao_a3/corregido/informe.xlsx
+++ b/examples/fao_a3/corregido/informe.xlsx
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>9217.581841240835</v>
+        <v>10084.81227148286</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>2.388462856078723</v>
+        <v>2.281080184364598</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>2304.395460310209</v>
+        <v>2521.203067870716</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>9217.581841240835</v>
+        <v>10084.81227148286</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2.388462856078723</v>
+        <v>2.281080184364598</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2.346599482965494</v>
+        <v>2.245097357179862</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1866,11 +1866,11 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3.129783917299089</v>
+        <v>2.989723140356754</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1, 1.5, 2, 2.5, 3</t>
+          <t>1, 1.5, 2, 2.5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -1887,11 +1887,11 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3.081435467889235</v>
+        <v>2.943492877017809</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1, 1.5, 2, 2.5, 3</t>
+          <t>1, 1.5, 2, 2.5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>warp_total_omits_doors: la resistencia total incluye ROB (Rem!H118 + D190)</t>
+          <t>warp_total_omits_doors: la resistencia total incluye ROB de los dos portones (Rem!H118 + 2·D190)</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
@@ -6484,7 +6484,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ROB portones [kgf]</t>
+          <t>ROB par de portones [kgf]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -6520,13 +6520,13 @@
         <v>1.356990427108308</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>17.69858020902099</v>
+        <v>35.39716041804198</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>421.7079375132039</v>
+        <v>439.4065177222249</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>434.951708587351</v>
+        <v>452.6502887963721</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>1395</v>
@@ -6549,13 +6549,13 @@
         <v>3.053228460993694</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>39.82180547029723</v>
+        <v>79.64361094059446</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>646.7792710454542</v>
+        <v>686.6010765157514</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>666.5817358541025</v>
+        <v>706.4035413243997</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>1342.5</v>
@@ -6578,13 +6578,13 @@
         <v>5.427961708433234</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>70.79432083608397</v>
+        <v>141.5886416721679</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>952.9140759446092</v>
+        <v>1023.708396780693</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>981.6020362353377</v>
+        <v>1052.396357071422</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>1290</v>
@@ -6607,13 +6607,13 @@
         <v>8.481190169426929</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>110.6161263063812</v>
+        <v>221.2322526127624</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>1334.285575858464</v>
+        <v>1444.901702164846</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1373.993011152582</v>
+        <v>1484.609137458963</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>1237.5</v>
@@ -6636,13 +6636,13 @@
         <v>12.21291384397478</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>159.2872218811889</v>
+        <v>318.5744437623778</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1787.099225051774</v>
+        <v>1946.386446932963</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>1839.788025521455</v>
+        <v>1999.075247402643</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>1185</v>
@@ -6665,13 +6665,13 @@
         <v>16.62313273207678</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>216.8076075605071</v>
+        <v>433.6152151210143</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>2304.395460310209</v>
+        <v>2521.203067870716</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>2371.87344601691</v>
+        <v>2588.681053577418</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>1132.5</v>
@@ -6694,13 +6694,13 @@
         <v>21.71184683373293</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>283.1772833443359</v>
+        <v>566.3545666886718</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>2882.969785094818</v>
+        <v>3166.147068439154</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>2966.90642692863</v>
+        <v>3250.083710272965</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>1080</v>
@@ -6723,13 +6723,13 @@
         <v>27.47905614894325</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>358.3962492326751</v>
+        <v>716.7924984653503</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>3519.057486821139</v>
+        <v>3877.453736053814</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>3620.997672160112</v>
+        <v>3979.393921392788</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1027.5</v>
@@ -6752,13 +6752,13 @@
         <v>33.92476067770772</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>442.4645052255249</v>
+        <v>884.9290104510497</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>4209.259347909127</v>
+        <v>4651.723853134651</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>4330.635475739494</v>
+        <v>4773.099980965018</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>975</v>
@@ -7241,7 +7241,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ROB hidrodinámica a 2 kn</t>
+          <t>ROB hidrodinámica de un portón a 2 kn</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ROB hidrodinámica a 3 kn</t>
+          <t>ROB hidrodinámica de un portón a 3 kn</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ROB hidrodinámica a 3.5 kn</t>
+          <t>ROB hidrodinámica de un portón a 3.5 kn</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">

</xml_diff>